<commit_message>
Update 2026 flume tank data
</commit_message>
<xml_diff>
--- a/analysis/flume_tank_2026/data/flume_tank_data_2026.xlsx
+++ b/analysis/flume_tank_2026/data/flume_tank_data_2026.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="529" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="495" uniqueCount="87">
   <si>
     <t>trial</t>
   </si>
@@ -101,10 +101,7 @@
     <t>A</t>
   </si>
   <si>
-    <t>PNE</t>
-  </si>
-  <si>
-    <t>1.2a</t>
+    <t>PNE (2026)</t>
   </si>
   <si>
     <t>EBS</t>
@@ -114,9 +111,6 @@
   </si>
   <si>
     <t>B</t>
-  </si>
-  <si>
-    <t>1.2b</t>
   </si>
   <si>
     <t>Rig B; 20" setback in the top, 10" in the middle, 20" bottom</t>
@@ -131,7 +125,7 @@
     <t>D</t>
   </si>
   <si>
-    <t>RACE</t>
+    <t>RACE (2026)</t>
   </si>
   <si>
     <t>GOA</t>
@@ -185,7 +179,7 @@
     <t>J</t>
   </si>
   <si>
-    <t>Standard</t>
+    <t>standard</t>
   </si>
   <si>
     <t>Rig J; 180' bridles, standard setback 18" top, 6" top; 0" footrope; middle bridle touching the bottom similar to the current PNE; no added weight on the bridles</t>
@@ -266,10 +260,16 @@
     <t>bottom_setback_links</t>
   </si>
   <si>
+    <t>PNE</t>
+  </si>
+  <si>
     <t>Rig A; Rigging prior to adjusting setback; height coming in low; 1 link middle (2.5"); 20" bottom setback</t>
   </si>
   <si>
     <t>Rig C; 20" setback in the top, 10" in the middle, 20" bottom; truncated bridles (sweeps 75 cm)</t>
+  </si>
+  <si>
+    <t>RACE</t>
   </si>
   <si>
     <t>Rig J; 180' bridles, standard setback 18" top, 6" middle; 0" footrope; middle bridle touching the bottom similar to the current PNE; no added weight on the bridles</t>
@@ -361,6 +361,9 @@
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" vertical="bottom"/>
@@ -370,9 +373,6 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
@@ -491,7 +491,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="D20:J23" displayName="Table_2" name="Table_2" id="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="D24:J27" displayName="Table_2" name="Table_2" id="2">
   <tableColumns count="7">
     <tableColumn name="Column1" id="1"/>
     <tableColumn name="Column2" id="2"/>
@@ -808,14 +808,14 @@
       <c r="C2" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D2" s="4" t="s">
-        <v>30</v>
+      <c r="D2" s="4">
+        <v>1.2</v>
       </c>
       <c r="E2" s="4">
         <v>27.9</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G2" s="5">
         <v>35.0</v>
@@ -881,7 +881,7 @@
         <v>22.6</v>
       </c>
       <c r="AB2" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3">
@@ -889,19 +889,19 @@
         <v>0.0</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D3" s="4" t="s">
-        <v>34</v>
+      <c r="D3" s="4">
+        <v>1.2</v>
       </c>
       <c r="E3" s="4">
         <v>27.9</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G3" s="5">
         <v>35.0</v>
@@ -967,7 +967,7 @@
         <v>22.8</v>
       </c>
       <c r="AB3" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4">
@@ -975,19 +975,19 @@
         <v>1.0</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D4" s="4" t="s">
-        <v>34</v>
+      <c r="D4" s="4">
+        <v>1.2</v>
       </c>
       <c r="E4" s="7">
         <v>27.9</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G4" s="5">
         <v>35.0</v>
@@ -1058,19 +1058,19 @@
         <v>2.0</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D5" s="4" t="s">
-        <v>34</v>
+      <c r="D5" s="4">
+        <v>1.2</v>
       </c>
       <c r="E5" s="5">
         <v>27.9</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G5" s="5">
         <v>35.0</v>
@@ -1142,19 +1142,19 @@
         <v>3.0</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D6" s="4" t="s">
-        <v>34</v>
+      <c r="D6" s="4">
+        <v>1.2</v>
       </c>
       <c r="E6" s="5">
         <v>27.9</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G6" s="5">
         <v>35.0</v>
@@ -1226,19 +1226,19 @@
         <v>4.0</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D7" s="4" t="s">
-        <v>34</v>
+      <c r="D7" s="4">
+        <v>1.2</v>
       </c>
       <c r="E7" s="5">
         <v>27.9</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G7" s="5">
         <v>35.0</v>
@@ -1310,19 +1310,19 @@
         <v>5.0</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D8" s="4" t="s">
-        <v>34</v>
+      <c r="D8" s="4">
+        <v>1.2</v>
       </c>
       <c r="E8" s="5">
         <v>27.9</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G8" s="5">
         <v>35.0</v>
@@ -1394,19 +1394,19 @@
         <v>6.0</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D9" s="4" t="s">
-        <v>34</v>
+      <c r="D9" s="4">
+        <v>1.2</v>
       </c>
       <c r="E9" s="5">
         <v>27.9</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G9" s="5">
         <v>35.0</v>
@@ -1478,19 +1478,19 @@
         <v>7.0</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D10" s="4" t="s">
-        <v>34</v>
+      <c r="D10" s="4">
+        <v>1.2</v>
       </c>
       <c r="E10" s="5">
         <v>27.9</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G10" s="5">
         <v>35.0</v>
@@ -1562,19 +1562,19 @@
         <v>8.0</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D11" s="4" t="s">
-        <v>34</v>
+      <c r="D11" s="4">
+        <v>1.2</v>
       </c>
       <c r="E11" s="5">
         <v>27.9</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G11" s="5">
         <v>35.0</v>
@@ -1646,19 +1646,19 @@
         <v>9.0</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D12" s="4" t="s">
-        <v>34</v>
+      <c r="D12" s="4">
+        <v>1.2</v>
       </c>
       <c r="E12" s="5">
         <v>27.9</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G12" s="5">
         <v>35.0</v>
@@ -1724,7 +1724,7 @@
         <v>30.5</v>
       </c>
       <c r="AB12" s="4" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="13">
@@ -1732,19 +1732,19 @@
         <v>10.0</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D13" s="4" t="s">
-        <v>34</v>
+      <c r="D13" s="4">
+        <v>1.2</v>
       </c>
       <c r="E13" s="5">
         <v>27.9</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G13" s="5">
         <v>35.0</v>
@@ -1816,19 +1816,19 @@
         <v>11.0</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D14" s="4" t="s">
-        <v>34</v>
+      <c r="D14" s="4">
+        <v>1.2</v>
       </c>
       <c r="E14" s="5">
         <v>27.9</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G14" s="5">
         <v>35.0</v>
@@ -1900,19 +1900,19 @@
         <v>12.0</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D15" s="4" t="s">
-        <v>34</v>
+      <c r="D15" s="4">
+        <v>1.2</v>
       </c>
       <c r="E15" s="5">
         <v>27.9</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G15" s="5">
         <v>35.0</v>
@@ -1984,19 +1984,19 @@
         <v>13.0</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D16" s="4" t="s">
-        <v>34</v>
+      <c r="D16" s="4">
+        <v>1.2</v>
       </c>
       <c r="E16" s="5">
         <v>27.9</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G16" s="5">
         <v>35.0</v>
@@ -2068,19 +2068,19 @@
         <v>14.0</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D17" s="4" t="s">
-        <v>34</v>
+      <c r="D17" s="4">
+        <v>1.2</v>
       </c>
       <c r="E17" s="5">
         <v>27.9</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G17" s="5">
         <v>35.0</v>
@@ -2152,19 +2152,19 @@
         <v>15.0</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D18" s="4" t="s">
-        <v>34</v>
+      <c r="D18" s="4">
+        <v>1.2</v>
       </c>
       <c r="E18" s="5">
         <v>27.9</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G18" s="5">
         <v>35.0</v>
@@ -2236,19 +2236,19 @@
         <v>16.0</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D19" s="4" t="s">
-        <v>34</v>
+      <c r="D19" s="4">
+        <v>1.2</v>
       </c>
       <c r="E19" s="5">
         <v>27.9</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G19" s="5">
         <v>35.0</v>
@@ -2320,10 +2320,10 @@
         <v>17.0</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D20" s="4">
         <v>1.0</v>
@@ -2332,7 +2332,7 @@
         <v>27.4</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G20" s="5">
         <v>34.0</v>
@@ -2398,7 +2398,7 @@
         <v>39.9</v>
       </c>
       <c r="AB20" s="4" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="21">
@@ -2406,10 +2406,10 @@
         <v>18.0</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D21" s="4">
         <v>1.0</v>
@@ -2418,7 +2418,7 @@
         <v>27.4</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G21" s="5">
         <v>34.0</v>
@@ -2484,7 +2484,7 @@
         <v>39.2</v>
       </c>
       <c r="AB21" s="4" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="22">
@@ -2492,10 +2492,10 @@
         <v>19.0</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D22" s="4">
         <v>1.0</v>
@@ -2504,7 +2504,7 @@
         <v>27.4</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G22" s="5">
         <v>34.0</v>
@@ -2570,7 +2570,7 @@
         <v>39.1</v>
       </c>
       <c r="AB22" s="4" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="23">
@@ -2578,10 +2578,10 @@
         <v>20.0</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D23" s="4">
         <v>1.0</v>
@@ -2590,7 +2590,7 @@
         <v>27.4</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G23" s="5">
         <v>34.0</v>
@@ -2656,7 +2656,7 @@
         <v>33.2</v>
       </c>
       <c r="AB23" s="4" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="24">
@@ -2664,10 +2664,10 @@
         <v>21.0</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D24" s="4">
         <v>1.0</v>
@@ -2676,7 +2676,7 @@
         <v>27.4</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G24" s="5">
         <v>34.0</v>
@@ -2748,10 +2748,10 @@
         <v>22.0</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D25" s="4">
         <v>1.0</v>
@@ -2760,7 +2760,7 @@
         <v>27.4</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G25" s="5">
         <v>34.0</v>
@@ -2832,10 +2832,10 @@
         <v>23.0</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D26" s="4">
         <v>1.0</v>
@@ -2844,7 +2844,7 @@
         <v>27.4</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G26" s="5">
         <v>34.0</v>
@@ -2916,10 +2916,10 @@
         <v>24.0</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D27" s="4">
         <v>1.0</v>
@@ -2928,7 +2928,7 @@
         <v>27.4</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G27" s="5">
         <v>34.0</v>
@@ -3000,10 +3000,10 @@
         <v>25.0</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D28" s="4">
         <v>1.0</v>
@@ -3012,7 +3012,7 @@
         <v>27.4</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G28" s="5">
         <v>34.0</v>
@@ -3078,7 +3078,7 @@
         <v>26.4</v>
       </c>
       <c r="AB28" s="4" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="29">
@@ -3086,10 +3086,10 @@
         <v>26.0</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D29" s="4">
         <v>1.0</v>
@@ -3098,7 +3098,7 @@
         <v>27.4</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G29" s="5">
         <v>34.0</v>
@@ -3170,10 +3170,10 @@
         <v>27.0</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D30" s="4">
         <v>1.0</v>
@@ -3182,7 +3182,7 @@
         <v>27.4</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G30" s="5">
         <v>34.0</v>
@@ -3253,10 +3253,10 @@
         <v>28.0</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D31" s="4">
         <v>1.0</v>
@@ -3265,7 +3265,7 @@
         <v>27.4</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G31" s="5">
         <v>34.0</v>
@@ -3337,10 +3337,10 @@
         <v>29.0</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D32" s="4">
         <v>1.0</v>
@@ -3349,7 +3349,7 @@
         <v>27.4</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G32" s="5">
         <v>34.0</v>
@@ -3421,10 +3421,10 @@
         <v>30.0</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D33" s="4">
         <v>1.0</v>
@@ -3433,7 +3433,7 @@
         <v>27.4</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G33" s="5">
         <v>34.0</v>
@@ -3505,10 +3505,10 @@
         <v>31.0</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D34" s="4">
         <v>1.0</v>
@@ -3517,7 +3517,7 @@
         <v>27.4</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G34" s="5">
         <v>34.0</v>
@@ -3589,10 +3589,10 @@
         <v>32.0</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D35" s="4">
         <v>1.0</v>
@@ -3601,7 +3601,7 @@
         <v>27.4</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G35" s="5">
         <v>34.0</v>
@@ -3673,10 +3673,10 @@
         <v>33.0</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D36" s="4">
         <v>1.0</v>
@@ -3685,7 +3685,7 @@
         <v>27.4</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G36" s="5">
         <v>34.0</v>
@@ -3751,7 +3751,7 @@
         <v>24.2</v>
       </c>
       <c r="AB36" s="4" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="37">
@@ -3759,10 +3759,10 @@
         <v>34.0</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D37" s="4">
         <v>1.0</v>
@@ -3771,7 +3771,7 @@
         <v>27.4</v>
       </c>
       <c r="F37" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G37" s="5">
         <v>34.0</v>
@@ -3837,7 +3837,7 @@
         <v>18.9</v>
       </c>
       <c r="AB37" s="4" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="38">
@@ -3845,10 +3845,10 @@
         <v>35.0</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D38" s="4">
         <v>1.0</v>
@@ -3857,7 +3857,7 @@
         <v>27.4</v>
       </c>
       <c r="F38" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G38" s="5">
         <v>34.0</v>
@@ -3929,10 +3929,10 @@
         <v>36.0</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D39" s="4">
         <v>1.0</v>
@@ -3941,7 +3941,7 @@
         <v>27.4</v>
       </c>
       <c r="F39" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G39" s="5">
         <v>34.0</v>
@@ -4007,7 +4007,7 @@
         <v>18.6</v>
       </c>
       <c r="AB39" s="4" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="40">
@@ -4015,10 +4015,10 @@
         <v>37.0</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D40" s="4">
         <v>1.0</v>
@@ -4027,7 +4027,7 @@
         <v>27.4</v>
       </c>
       <c r="F40" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G40" s="5">
         <v>34.0</v>
@@ -4099,10 +4099,10 @@
         <v>38.0</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D41" s="4">
         <v>1.0</v>
@@ -4111,7 +4111,7 @@
         <v>27.4</v>
       </c>
       <c r="F41" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G41" s="5">
         <v>34.0</v>
@@ -4183,10 +4183,10 @@
         <v>39.0</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D42" s="4">
         <v>1.0</v>
@@ -4195,7 +4195,7 @@
         <v>27.4</v>
       </c>
       <c r="F42" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G42" s="5">
         <v>34.0</v>
@@ -4267,10 +4267,10 @@
         <v>40.0</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D43" s="4">
         <v>1.0</v>
@@ -4279,7 +4279,7 @@
         <v>27.4</v>
       </c>
       <c r="F43" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G43" s="5">
         <v>34.0</v>
@@ -4351,10 +4351,10 @@
         <v>41.0</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D44" s="4">
         <v>1.0</v>
@@ -4363,7 +4363,7 @@
         <v>27.4</v>
       </c>
       <c r="F44" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G44" s="5">
         <v>34.0</v>
@@ -4435,10 +4435,10 @@
         <v>42.0</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D45" s="4">
         <v>1.0</v>
@@ -4447,7 +4447,7 @@
         <v>27.4</v>
       </c>
       <c r="F45" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G45" s="5">
         <v>34.0</v>
@@ -4513,7 +4513,7 @@
         <v>32.6</v>
       </c>
       <c r="AB45" s="4" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="46">
@@ -4521,10 +4521,10 @@
         <v>43.0</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D46" s="4">
         <v>1.0</v>
@@ -4533,7 +4533,7 @@
         <v>27.4</v>
       </c>
       <c r="F46" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G46" s="5">
         <v>34.0</v>
@@ -4605,10 +4605,10 @@
         <v>44.0</v>
       </c>
       <c r="B47" s="4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D47" s="4">
         <v>1.0</v>
@@ -4617,7 +4617,7 @@
         <v>27.4</v>
       </c>
       <c r="F47" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G47" s="5">
         <v>34.0</v>
@@ -4689,10 +4689,10 @@
         <v>45.0</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D48" s="4">
         <v>1.0</v>
@@ -4701,7 +4701,7 @@
         <v>27.4</v>
       </c>
       <c r="F48" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G48" s="5">
         <v>34.0</v>
@@ -4773,10 +4773,10 @@
         <v>46.0</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D49" s="4">
         <v>1.0</v>
@@ -4785,7 +4785,7 @@
         <v>27.4</v>
       </c>
       <c r="F49" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G49" s="5">
         <v>34.0</v>
@@ -4857,19 +4857,19 @@
         <v>47.0</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D50" s="4" t="s">
-        <v>34</v>
+        <v>37</v>
+      </c>
+      <c r="D50" s="4">
+        <v>1.2</v>
       </c>
       <c r="E50" s="5">
         <v>27.8</v>
       </c>
       <c r="F50" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G50" s="5">
         <v>34.0</v>
@@ -4935,7 +4935,7 @@
         <v>26.8</v>
       </c>
       <c r="AB50" s="4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="51">
@@ -4943,19 +4943,19 @@
         <v>48.0</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D51" s="4" t="s">
-        <v>34</v>
+        <v>37</v>
+      </c>
+      <c r="D51" s="4">
+        <v>1.2</v>
       </c>
       <c r="E51" s="5">
         <v>27.8</v>
       </c>
       <c r="F51" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G51" s="5">
         <v>34.0</v>
@@ -5021,7 +5021,7 @@
         <v>26.1</v>
       </c>
       <c r="AB51" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="52">
@@ -5029,19 +5029,19 @@
         <v>49.0</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D52" s="4" t="s">
-        <v>34</v>
+        <v>37</v>
+      </c>
+      <c r="D52" s="4">
+        <v>1.2</v>
       </c>
       <c r="E52" s="5">
         <v>27.8</v>
       </c>
       <c r="F52" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G52" s="5">
         <v>34.0</v>
@@ -5107,7 +5107,7 @@
         <v>25.6</v>
       </c>
       <c r="AB52" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="53">
@@ -5115,19 +5115,19 @@
         <v>50.0</v>
       </c>
       <c r="B53" s="4" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D53" s="4" t="s">
-        <v>34</v>
+        <v>37</v>
+      </c>
+      <c r="D53" s="4">
+        <v>1.2</v>
       </c>
       <c r="E53" s="5">
         <v>27.8</v>
       </c>
       <c r="F53" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G53" s="5">
         <v>34.0</v>
@@ -5193,7 +5193,7 @@
         <v>30.5</v>
       </c>
       <c r="AB53" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="54">
@@ -5201,19 +5201,19 @@
         <v>51.0</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D54" s="4" t="s">
-        <v>34</v>
+        <v>37</v>
+      </c>
+      <c r="D54" s="4">
+        <v>1.2</v>
       </c>
       <c r="E54" s="5">
         <v>27.8</v>
       </c>
       <c r="F54" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G54" s="5">
         <v>34.0</v>
@@ -5279,7 +5279,7 @@
         <v>30.8</v>
       </c>
       <c r="AB54" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="55">
@@ -5287,19 +5287,19 @@
         <v>52.0</v>
       </c>
       <c r="B55" s="4" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D55" s="4" t="s">
-        <v>34</v>
+        <v>37</v>
+      </c>
+      <c r="D55" s="4">
+        <v>1.2</v>
       </c>
       <c r="E55" s="5">
         <v>27.8</v>
       </c>
       <c r="F55" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G55" s="5">
         <v>34.0</v>
@@ -5365,7 +5365,7 @@
         <v>30.7</v>
       </c>
       <c r="AB55" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="56">
@@ -5373,19 +5373,19 @@
         <v>53.0</v>
       </c>
       <c r="B56" s="4" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D56" s="4" t="s">
-        <v>34</v>
+        <v>37</v>
+      </c>
+      <c r="D56" s="4">
+        <v>1.2</v>
       </c>
       <c r="E56" s="5">
         <v>27.8</v>
       </c>
       <c r="F56" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G56" s="5">
         <v>34.0</v>
@@ -5451,7 +5451,7 @@
         <v>24.4</v>
       </c>
       <c r="AB56" s="4" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="57">
@@ -5459,19 +5459,19 @@
         <v>54.0</v>
       </c>
       <c r="B57" s="4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C57" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D57" s="4" t="s">
-        <v>34</v>
+      <c r="D57" s="4">
+        <v>1.2</v>
       </c>
       <c r="E57" s="5">
         <v>27.9</v>
       </c>
       <c r="F57" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G57" s="5">
         <v>35.0</v>
@@ -5537,7 +5537,7 @@
         <v>35.8</v>
       </c>
       <c r="AB57" s="4" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="58">
@@ -5545,19 +5545,19 @@
         <v>55.0</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C58" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D58" s="4" t="s">
-        <v>34</v>
+      <c r="D58" s="4">
+        <v>1.2</v>
       </c>
       <c r="E58" s="5">
         <v>27.9</v>
       </c>
       <c r="F58" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G58" s="5">
         <v>35.0</v>
@@ -5629,19 +5629,19 @@
         <v>56.0</v>
       </c>
       <c r="B59" s="4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C59" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D59" s="4" t="s">
-        <v>34</v>
+      <c r="D59" s="4">
+        <v>1.2</v>
       </c>
       <c r="E59" s="5">
         <v>27.9</v>
       </c>
       <c r="F59" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G59" s="5">
         <v>35.0</v>
@@ -5713,19 +5713,19 @@
         <v>57.0</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C60" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D60" s="4" t="s">
-        <v>34</v>
+      <c r="D60" s="4">
+        <v>1.2</v>
       </c>
       <c r="E60" s="5">
         <v>27.9</v>
       </c>
       <c r="F60" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G60" s="5">
         <v>35.0</v>
@@ -5797,19 +5797,19 @@
         <v>58.0</v>
       </c>
       <c r="B61" s="4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C61" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D61" s="4" t="s">
-        <v>34</v>
+      <c r="D61" s="4">
+        <v>1.2</v>
       </c>
       <c r="E61" s="5">
         <v>27.9</v>
       </c>
       <c r="F61" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G61" s="5">
         <v>35.0</v>
@@ -5881,19 +5881,19 @@
         <v>59.0</v>
       </c>
       <c r="B62" s="4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C62" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D62" s="4" t="s">
-        <v>34</v>
+      <c r="D62" s="4">
+        <v>1.2</v>
       </c>
       <c r="E62" s="5">
         <v>27.9</v>
       </c>
       <c r="F62" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G62" s="5">
         <v>35.0</v>
@@ -5965,19 +5965,19 @@
         <v>60.0</v>
       </c>
       <c r="B63" s="4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C63" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D63" s="4" t="s">
-        <v>34</v>
+      <c r="D63" s="4">
+        <v>1.2</v>
       </c>
       <c r="E63" s="5">
         <v>27.9</v>
       </c>
       <c r="F63" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G63" s="5">
         <v>35.0</v>
@@ -6049,19 +6049,19 @@
         <v>61.0</v>
       </c>
       <c r="B64" s="4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C64" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D64" s="4" t="s">
-        <v>34</v>
+      <c r="D64" s="4">
+        <v>1.2</v>
       </c>
       <c r="E64" s="5">
         <v>27.9</v>
       </c>
       <c r="F64" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G64" s="5">
         <v>35.0</v>
@@ -6133,19 +6133,19 @@
         <v>62.0</v>
       </c>
       <c r="B65" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C65" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D65" s="4" t="s">
-        <v>34</v>
+      <c r="D65" s="4">
+        <v>1.2</v>
       </c>
       <c r="E65" s="5">
         <v>27.9</v>
       </c>
       <c r="F65" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G65" s="5">
         <v>35.0</v>
@@ -6211,7 +6211,7 @@
         <v>22.4</v>
       </c>
       <c r="AB65" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="66">
@@ -6219,19 +6219,19 @@
         <v>63.0</v>
       </c>
       <c r="B66" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C66" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D66" s="4" t="s">
-        <v>34</v>
+      <c r="D66" s="4">
+        <v>1.2</v>
       </c>
       <c r="E66" s="5">
         <v>27.9</v>
       </c>
       <c r="F66" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G66" s="5">
         <v>35.0</v>
@@ -6303,19 +6303,19 @@
         <v>64.0</v>
       </c>
       <c r="B67" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C67" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D67" s="4" t="s">
-        <v>34</v>
+      <c r="D67" s="4">
+        <v>1.2</v>
       </c>
       <c r="E67" s="5">
         <v>27.9</v>
       </c>
       <c r="F67" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G67" s="5">
         <v>35.0</v>
@@ -6387,19 +6387,19 @@
         <v>65.0</v>
       </c>
       <c r="B68" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C68" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D68" s="4" t="s">
-        <v>34</v>
+      <c r="D68" s="4">
+        <v>1.2</v>
       </c>
       <c r="E68" s="5">
         <v>27.9</v>
       </c>
       <c r="F68" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G68" s="5">
         <v>35.0</v>
@@ -6471,19 +6471,19 @@
         <v>66.0</v>
       </c>
       <c r="B69" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C69" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D69" s="4" t="s">
-        <v>34</v>
+      <c r="D69" s="4">
+        <v>1.2</v>
       </c>
       <c r="E69" s="5">
         <v>27.9</v>
       </c>
       <c r="F69" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G69" s="5">
         <v>35.0</v>
@@ -6555,19 +6555,19 @@
         <v>67.0</v>
       </c>
       <c r="B70" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C70" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D70" s="4" t="s">
-        <v>34</v>
+      <c r="D70" s="4">
+        <v>1.2</v>
       </c>
       <c r="E70" s="5">
         <v>27.9</v>
       </c>
       <c r="F70" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G70" s="5">
         <v>35.0</v>
@@ -6633,7 +6633,7 @@
         <v>17.6</v>
       </c>
       <c r="AB70" s="4" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="71">
@@ -6641,19 +6641,19 @@
         <v>68.0</v>
       </c>
       <c r="B71" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C71" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D71" s="4" t="s">
-        <v>34</v>
+      <c r="D71" s="4">
+        <v>1.2</v>
       </c>
       <c r="E71" s="5">
         <v>27.9</v>
       </c>
       <c r="F71" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G71" s="5">
         <v>35.0</v>
@@ -6725,19 +6725,19 @@
         <v>69.0</v>
       </c>
       <c r="B72" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C72" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D72" s="4" t="s">
-        <v>34</v>
+      <c r="D72" s="4">
+        <v>1.2</v>
       </c>
       <c r="E72" s="5">
         <v>27.9</v>
       </c>
       <c r="F72" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G72" s="5">
         <v>35.0</v>
@@ -6809,19 +6809,19 @@
         <v>70.0</v>
       </c>
       <c r="B73" s="4" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C73" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D73" s="4" t="s">
-        <v>57</v>
+      <c r="D73" s="9" t="s">
+        <v>55</v>
       </c>
       <c r="E73" s="5">
         <v>27.9</v>
       </c>
       <c r="F73" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G73" s="5">
         <v>35.0</v>
@@ -6887,7 +6887,7 @@
         <v>22.7</v>
       </c>
       <c r="AB73" s="4" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="74">
@@ -6895,19 +6895,19 @@
         <v>71.0</v>
       </c>
       <c r="B74" s="4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C74" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D74" s="4" t="s">
-        <v>57</v>
+      <c r="D74" s="9" t="s">
+        <v>55</v>
       </c>
       <c r="E74" s="5">
         <v>28.0</v>
       </c>
       <c r="F74" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G74" s="5">
         <v>35.0</v>
@@ -6973,7 +6973,7 @@
         <v>22.8</v>
       </c>
       <c r="AB74" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="75">
@@ -6981,19 +6981,19 @@
         <v>72.0</v>
       </c>
       <c r="B75" s="4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C75" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D75" s="4" t="s">
-        <v>57</v>
+      <c r="D75" s="9" t="s">
+        <v>55</v>
       </c>
       <c r="E75" s="5">
         <v>28.0</v>
       </c>
       <c r="F75" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G75" s="5">
         <v>35.0</v>
@@ -7065,19 +7065,19 @@
         <v>73.0</v>
       </c>
       <c r="B76" s="4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C76" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D76" s="4" t="s">
-        <v>57</v>
+      <c r="D76" s="9" t="s">
+        <v>55</v>
       </c>
       <c r="E76" s="5">
         <v>28.0</v>
       </c>
       <c r="F76" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G76" s="5">
         <v>35.0</v>
@@ -7149,19 +7149,19 @@
         <v>74.0</v>
       </c>
       <c r="B77" s="4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C77" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D77" s="4" t="s">
-        <v>57</v>
+        <v>37</v>
+      </c>
+      <c r="D77" s="9" t="s">
+        <v>55</v>
       </c>
       <c r="E77" s="5">
         <v>28.0</v>
       </c>
       <c r="F77" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G77" s="5">
         <v>34.0</v>
@@ -7227,7 +7227,7 @@
         <v>24.4</v>
       </c>
       <c r="AB77" s="4" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="78">
@@ -7235,19 +7235,19 @@
         <v>75.0</v>
       </c>
       <c r="B78" s="4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C78" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D78" s="4" t="s">
-        <v>57</v>
+        <v>37</v>
+      </c>
+      <c r="D78" s="9" t="s">
+        <v>55</v>
       </c>
       <c r="E78" s="5">
         <v>28.0</v>
       </c>
       <c r="F78" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G78" s="5">
         <v>34.0</v>
@@ -7319,19 +7319,19 @@
         <v>76.0</v>
       </c>
       <c r="B79" s="4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C79" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D79" s="4" t="s">
-        <v>57</v>
+        <v>37</v>
+      </c>
+      <c r="D79" s="9" t="s">
+        <v>55</v>
       </c>
       <c r="E79" s="5">
         <v>28.0</v>
       </c>
       <c r="F79" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G79" s="5">
         <v>34.0</v>
@@ -7397,7 +7397,7 @@
         <v>24.1</v>
       </c>
       <c r="AB79" s="4" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="80">
@@ -7405,19 +7405,19 @@
         <v>77.0</v>
       </c>
       <c r="B80" s="4" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C80" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D80" s="4" t="s">
-        <v>57</v>
+        <v>37</v>
+      </c>
+      <c r="D80" s="9" t="s">
+        <v>55</v>
       </c>
       <c r="E80" s="5">
         <v>28.0</v>
       </c>
       <c r="F80" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G80" s="5">
         <v>34.0</v>
@@ -7475,7 +7475,7 @@
         <v>23.5</v>
       </c>
       <c r="AB80" s="4" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="81">
@@ -7483,19 +7483,19 @@
         <v>78.0</v>
       </c>
       <c r="B81" s="4" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C81" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D81" s="4" t="s">
-        <v>57</v>
+        <v>37</v>
+      </c>
+      <c r="D81" s="9" t="s">
+        <v>55</v>
       </c>
       <c r="E81" s="5">
         <v>26.1</v>
       </c>
       <c r="F81" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G81" s="5">
         <v>34.0</v>
@@ -7559,19 +7559,19 @@
         <v>79.0</v>
       </c>
       <c r="B82" s="4" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C82" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D82" s="4" t="s">
-        <v>57</v>
+        <v>37</v>
+      </c>
+      <c r="D82" s="9" t="s">
+        <v>55</v>
       </c>
       <c r="E82" s="5">
         <v>28.0</v>
       </c>
       <c r="F82" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G82" s="5">
         <v>34.0</v>
@@ -7635,19 +7635,19 @@
         <v>80.0</v>
       </c>
       <c r="B83" s="4" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C83" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D83" s="4" t="s">
-        <v>57</v>
+        <v>37</v>
+      </c>
+      <c r="D83" s="9" t="s">
+        <v>55</v>
       </c>
       <c r="E83" s="5">
         <v>28.0</v>
       </c>
       <c r="F83" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G83" s="5">
         <v>34.0</v>
@@ -7711,19 +7711,19 @@
         <v>81.0</v>
       </c>
       <c r="B84" s="4" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C84" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D84" s="4" t="s">
-        <v>57</v>
+        <v>37</v>
+      </c>
+      <c r="D84" s="9" t="s">
+        <v>55</v>
       </c>
       <c r="E84" s="5">
         <v>28.0</v>
       </c>
       <c r="F84" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G84" s="5">
         <v>34.0</v>
@@ -7787,19 +7787,19 @@
         <v>82.0</v>
       </c>
       <c r="B85" s="4" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C85" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D85" s="4" t="s">
-        <v>57</v>
+        <v>37</v>
+      </c>
+      <c r="D85" s="9" t="s">
+        <v>55</v>
       </c>
       <c r="E85" s="5">
         <v>28.0</v>
       </c>
       <c r="F85" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G85" s="5">
         <v>34.0</v>
@@ -7863,19 +7863,19 @@
         <v>83.0</v>
       </c>
       <c r="B86" s="4" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C86" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D86" s="4" t="s">
-        <v>57</v>
+      <c r="D86" s="9" t="s">
+        <v>55</v>
       </c>
       <c r="E86" s="5">
         <v>26.1</v>
       </c>
       <c r="F86" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G86" s="5">
         <v>35.0</v>
@@ -7896,7 +7896,7 @@
       <c r="M86" s="4">
         <v>16.0</v>
       </c>
-      <c r="N86" s="9">
+      <c r="N86" s="10">
         <f t="shared" ref="N86:N87" si="19">2.01*8</f>
         <v>16.08</v>
       </c>
@@ -7909,7 +7909,7 @@
       <c r="Q86" s="6">
         <v>17.9</v>
       </c>
-      <c r="R86" s="9">
+      <c r="R86" s="10">
         <f>0.884*8</f>
         <v>7.072</v>
       </c>
@@ -7939,19 +7939,19 @@
         <v>84.0</v>
       </c>
       <c r="B87" s="4" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C87" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D87" s="4" t="s">
-        <v>57</v>
+      <c r="D87" s="9" t="s">
+        <v>55</v>
       </c>
       <c r="E87" s="5">
         <v>26.1</v>
       </c>
       <c r="F87" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G87" s="5">
         <v>35.0</v>
@@ -8015,19 +8015,19 @@
         <v>85.0</v>
       </c>
       <c r="B88" s="4" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C88" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D88" s="4" t="s">
-        <v>57</v>
+      <c r="D88" s="9" t="s">
+        <v>55</v>
       </c>
       <c r="E88" s="5">
         <v>26.1</v>
       </c>
       <c r="F88" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G88" s="5">
         <v>35.0</v>
@@ -8091,19 +8091,19 @@
         <v>86.0</v>
       </c>
       <c r="B89" s="4" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C89" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D89" s="4" t="s">
-        <v>57</v>
+      <c r="D89" s="9" t="s">
+        <v>55</v>
       </c>
       <c r="E89" s="5">
         <v>26.1</v>
       </c>
       <c r="F89" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G89" s="5">
         <v>35.0</v>
@@ -8167,19 +8167,19 @@
         <v>87.0</v>
       </c>
       <c r="B90" s="4" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C90" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D90" s="4" t="s">
-        <v>57</v>
+      <c r="D90" s="9" t="s">
+        <v>55</v>
       </c>
       <c r="E90" s="5">
         <v>26.1</v>
       </c>
       <c r="F90" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G90" s="5">
         <v>35.0</v>
@@ -8243,19 +8243,19 @@
         <v>88.0</v>
       </c>
       <c r="B91" s="4" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C91" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D91" s="4" t="s">
-        <v>57</v>
+      <c r="D91" s="9" t="s">
+        <v>55</v>
       </c>
       <c r="E91" s="5">
         <v>26.1</v>
       </c>
       <c r="F91" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G91" s="5">
         <v>35.0</v>
@@ -8319,19 +8319,19 @@
         <v>89.0</v>
       </c>
       <c r="B92" s="4" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C92" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D92" s="4" t="s">
-        <v>34</v>
+      <c r="D92" s="4">
+        <v>1.2</v>
       </c>
       <c r="E92" s="5">
         <v>27.9</v>
       </c>
       <c r="F92" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G92" s="5">
         <v>47.0</v>
@@ -8397,7 +8397,7 @@
         <v>21.6</v>
       </c>
       <c r="AB92" s="4" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="93">
@@ -8405,19 +8405,19 @@
         <v>90.0</v>
       </c>
       <c r="B93" s="4" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C93" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D93" s="4" t="s">
-        <v>34</v>
+      <c r="D93" s="4">
+        <v>1.2</v>
       </c>
       <c r="E93" s="5">
         <v>27.9</v>
       </c>
       <c r="F93" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G93" s="5">
         <v>47.0</v>
@@ -8483,7 +8483,7 @@
         <v>21.8</v>
       </c>
       <c r="AB93" s="4" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="94">
@@ -8491,7 +8491,7 @@
         <v>91.0</v>
       </c>
       <c r="B94" s="4" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C94" s="4" t="s">
         <v>29</v>
@@ -8503,7 +8503,7 @@
         <v>27.9</v>
       </c>
       <c r="F94" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G94" s="5">
         <v>47.0</v>
@@ -8569,7 +8569,7 @@
         <v>22.5</v>
       </c>
       <c r="AB94" s="4" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="95">
@@ -8577,7 +8577,7 @@
         <v>92.0</v>
       </c>
       <c r="B95" s="4" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C95" s="4" t="s">
         <v>29</v>
@@ -8585,17 +8585,17 @@
       <c r="D95" s="4">
         <v>2.0</v>
       </c>
-      <c r="E95" s="10">
+      <c r="E95" s="11">
         <v>27.9</v>
       </c>
       <c r="F95" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="G95" s="11"/>
-      <c r="H95" s="11"/>
+        <v>38</v>
+      </c>
+      <c r="G95" s="12"/>
+      <c r="H95" s="12"/>
       <c r="I95" s="6"/>
-      <c r="J95" s="11"/>
-      <c r="K95" s="11"/>
+      <c r="J95" s="12"/>
+      <c r="K95" s="12"/>
       <c r="L95" s="4">
         <v>3.0</v>
       </c>
@@ -8606,24 +8606,24 @@
         <f>1.99*8</f>
         <v>15.92</v>
       </c>
-      <c r="O95" s="11"/>
-      <c r="P95" s="11"/>
+      <c r="O95" s="12"/>
+      <c r="P95" s="12"/>
       <c r="Q95" s="6"/>
       <c r="R95" s="6">
         <f>0.593*8</f>
         <v>4.744</v>
       </c>
-      <c r="S95" s="11"/>
-      <c r="T95" s="11"/>
-      <c r="U95" s="11"/>
-      <c r="V95" s="11"/>
-      <c r="W95" s="11"/>
-      <c r="X95" s="11"/>
-      <c r="Y95" s="11"/>
-      <c r="Z95" s="11"/>
-      <c r="AA95" s="12"/>
+      <c r="S95" s="12"/>
+      <c r="T95" s="12"/>
+      <c r="U95" s="12"/>
+      <c r="V95" s="12"/>
+      <c r="W95" s="12"/>
+      <c r="X95" s="12"/>
+      <c r="Y95" s="12"/>
+      <c r="Z95" s="12"/>
+      <c r="AA95" s="13"/>
       <c r="AB95" s="4" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="96">
@@ -8631,10 +8631,10 @@
         <v>93.0</v>
       </c>
       <c r="B96" s="4" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C96" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D96" s="4">
         <v>2.0</v>
@@ -8643,7 +8643,7 @@
         <v>27.9</v>
       </c>
       <c r="F96" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G96" s="5">
         <v>47.0</v>
@@ -8709,7 +8709,7 @@
         <v>21.8</v>
       </c>
       <c r="AB96" s="4" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="97">
@@ -8717,10 +8717,10 @@
         <v>94.0</v>
       </c>
       <c r="B97" s="4" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C97" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D97" s="4">
         <v>2.0</v>
@@ -8729,7 +8729,7 @@
         <v>27.9</v>
       </c>
       <c r="F97" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G97" s="5">
         <v>47.0</v>
@@ -8795,7 +8795,7 @@
         <v>22.5</v>
       </c>
       <c r="AB97" s="4" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="98">
@@ -8803,10 +8803,10 @@
         <v>95.0</v>
       </c>
       <c r="B98" s="4" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C98" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D98" s="4">
         <v>1.0</v>
@@ -8815,7 +8815,7 @@
         <v>27.4</v>
       </c>
       <c r="F98" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G98" s="5">
         <v>47.0</v>
@@ -8881,7 +8881,7 @@
         <v>23.4</v>
       </c>
       <c r="AB98" s="4" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="99">
@@ -8889,10 +8889,10 @@
         <v>96.0</v>
       </c>
       <c r="B99" s="4" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C99" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D99" s="4">
         <v>1.0</v>
@@ -8901,7 +8901,7 @@
         <v>27.4</v>
       </c>
       <c r="F99" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G99" s="5">
         <v>47.0</v>
@@ -8967,7 +8967,7 @@
         <v>23.4</v>
       </c>
       <c r="AB99" s="4" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
   </sheetData>
@@ -8992,739 +8992,867 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="C1" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="D1" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="13" t="s">
+      <c r="E1" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="13" t="s">
+      <c r="F1" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="G1" s="13" t="s">
+      <c r="G1" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="H1" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="I1" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="H1" s="13" t="s">
+      <c r="J1" s="9" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="B2" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="I1" s="13" t="s">
+      <c r="C2" s="9">
+        <v>1.2</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="E2" s="9">
+        <v>3.43</v>
+      </c>
+      <c r="F2" s="9">
+        <v>3.43</v>
+      </c>
+      <c r="G2" s="9">
+        <v>8.0</v>
+      </c>
+      <c r="H2" s="9">
+        <v>1.0</v>
+      </c>
+      <c r="I2" s="9">
+        <v>8.0</v>
+      </c>
+      <c r="J2" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="J1" s="13" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="B2" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="C2" s="13" t="s">
+    </row>
+    <row r="3">
+      <c r="A3" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="C3" s="9">
+        <v>1.2</v>
+      </c>
+      <c r="D3" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="D2" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="E2" s="13">
+      <c r="E3" s="9">
         <v>3.43</v>
       </c>
-      <c r="F2" s="13">
+      <c r="F3" s="9">
         <v>3.43</v>
       </c>
-      <c r="G2" s="13">
+      <c r="G3" s="9">
         <v>8.0</v>
       </c>
-      <c r="H2" s="13">
-        <v>1.0</v>
-      </c>
-      <c r="I2" s="13">
+      <c r="H3" s="9">
+        <v>4.0</v>
+      </c>
+      <c r="I3" s="9">
         <v>8.0</v>
       </c>
-      <c r="J2" s="13" t="s">
+      <c r="J3" s="9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="C4" s="9">
+        <v>1.2</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="E4" s="9">
+        <v>3.43</v>
+      </c>
+      <c r="F4" s="9">
+        <v>3.43</v>
+      </c>
+      <c r="G4" s="9">
+        <v>8.0</v>
+      </c>
+      <c r="H4" s="9">
+        <v>4.0</v>
+      </c>
+      <c r="I4" s="9">
+        <v>8.0</v>
+      </c>
+      <c r="J4" s="9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="C5" s="9">
+        <v>1.2</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="E5" s="9">
+        <v>3.43</v>
+      </c>
+      <c r="F5" s="9">
+        <v>0.75</v>
+      </c>
+      <c r="G5" s="9">
+        <v>8.0</v>
+      </c>
+      <c r="H5" s="9">
+        <v>4.0</v>
+      </c>
+      <c r="I5" s="9">
+        <v>8.0</v>
+      </c>
+      <c r="J5" s="9" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="13" t="s">
-        <v>33</v>
-      </c>
-      <c r="B3" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="C3" s="13" t="s">
+    <row r="6">
+      <c r="A6" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="D3" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="E3" s="13">
+      <c r="B6" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="C6" s="9">
+        <v>1.2</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="E6" s="9">
         <v>3.43</v>
       </c>
-      <c r="F3" s="13">
-        <v>3.43</v>
-      </c>
-      <c r="G3" s="13">
+      <c r="F6" s="9">
+        <v>0.75</v>
+      </c>
+      <c r="G6" s="9">
         <v>8.0</v>
       </c>
-      <c r="H3" s="13">
+      <c r="H6" s="9">
         <v>4.0</v>
       </c>
-      <c r="I3" s="13">
+      <c r="I6" s="9">
         <v>8.0</v>
       </c>
-      <c r="J3" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="13" t="s">
+      <c r="J6" s="9" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="B4" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="C4" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="D4" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="E4" s="13">
-        <v>3.43</v>
-      </c>
-      <c r="F4" s="13">
-        <v>0.75</v>
-      </c>
-      <c r="G4" s="13">
-        <v>8.0</v>
-      </c>
-      <c r="H4" s="13">
-        <v>4.0</v>
-      </c>
-      <c r="I4" s="13">
-        <v>8.0</v>
-      </c>
-      <c r="J4" s="13" t="s">
+      <c r="B7" s="9" t="s">
         <v>85</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="13" t="s">
-        <v>38</v>
-      </c>
-      <c r="B5" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="C5" s="14">
-        <v>1.0</v>
-      </c>
-      <c r="D5" s="13" t="s">
-        <v>40</v>
-      </c>
-      <c r="E5" s="13">
-        <v>3.43</v>
-      </c>
-      <c r="F5" s="13">
-        <v>0.5</v>
-      </c>
-      <c r="G5" s="13">
-        <v>0.0</v>
-      </c>
-      <c r="H5" s="13">
-        <v>0.0</v>
-      </c>
-      <c r="I5" s="13">
-        <v>0.0</v>
-      </c>
-      <c r="J5" s="13" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="13" t="s">
-        <v>43</v>
-      </c>
-      <c r="B6" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="C6" s="14">
-        <v>1.0</v>
-      </c>
-      <c r="D6" s="13" t="s">
-        <v>40</v>
-      </c>
-      <c r="E6" s="13">
-        <v>3.43</v>
-      </c>
-      <c r="F6" s="13">
-        <v>0.75</v>
-      </c>
-      <c r="G6" s="13">
-        <v>0.0</v>
-      </c>
-      <c r="H6" s="13">
-        <v>0.0</v>
-      </c>
-      <c r="I6" s="13">
-        <v>0.0</v>
-      </c>
-      <c r="J6" s="13" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="B7" s="13" t="s">
-        <v>39</v>
       </c>
       <c r="C7" s="14">
         <v>1.0</v>
       </c>
-      <c r="D7" s="13" t="s">
-        <v>40</v>
-      </c>
-      <c r="E7" s="13">
+      <c r="D7" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="E7" s="9">
         <v>3.43</v>
       </c>
-      <c r="F7" s="13">
-        <v>3.43</v>
-      </c>
-      <c r="G7" s="13">
-        <v>0.0</v>
-      </c>
-      <c r="H7" s="13">
-        <v>0.0</v>
-      </c>
-      <c r="I7" s="13">
-        <v>0.0</v>
-      </c>
-      <c r="J7" s="13" t="s">
-        <v>48</v>
+      <c r="F7" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="G7" s="9">
+        <v>0.0</v>
+      </c>
+      <c r="H7" s="9">
+        <v>0.0</v>
+      </c>
+      <c r="I7" s="9">
+        <v>0.0</v>
+      </c>
+      <c r="J7" s="9" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="s">
-        <v>45</v>
-      </c>
-      <c r="B8" s="13" t="s">
-        <v>39</v>
+      <c r="A8" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>85</v>
       </c>
       <c r="C8" s="14">
         <v>1.0</v>
       </c>
-      <c r="D8" s="13" t="s">
-        <v>40</v>
-      </c>
-      <c r="E8" s="13">
+      <c r="D8" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="E8" s="9">
         <v>3.43</v>
       </c>
-      <c r="F8" s="13">
+      <c r="F8" s="9">
+        <v>0.75</v>
+      </c>
+      <c r="G8" s="9">
+        <v>0.0</v>
+      </c>
+      <c r="H8" s="9">
+        <v>0.0</v>
+      </c>
+      <c r="I8" s="9">
+        <v>0.0</v>
+      </c>
+      <c r="J8" s="9" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="C9" s="14">
+        <v>1.0</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="E9" s="9">
+        <v>3.43</v>
+      </c>
+      <c r="F9" s="9">
+        <v>0.75</v>
+      </c>
+      <c r="G9" s="9">
+        <v>0.0</v>
+      </c>
+      <c r="H9" s="9">
+        <v>0.0</v>
+      </c>
+      <c r="I9" s="9">
+        <v>0.0</v>
+      </c>
+      <c r="J9" s="9" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="C10" s="14">
+        <v>1.0</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="E10" s="9">
+        <v>3.43</v>
+      </c>
+      <c r="F10" s="9">
+        <v>3.43</v>
+      </c>
+      <c r="G10" s="9">
+        <v>0.0</v>
+      </c>
+      <c r="H10" s="9">
+        <v>0.0</v>
+      </c>
+      <c r="I10" s="9">
+        <v>0.0</v>
+      </c>
+      <c r="J10" s="9" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="C11" s="14">
+        <v>1.0</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="E11" s="9">
+        <v>3.43</v>
+      </c>
+      <c r="F11" s="9">
+        <v>3.43</v>
+      </c>
+      <c r="G11" s="9">
+        <v>0.0</v>
+      </c>
+      <c r="H11" s="9">
+        <v>0.0</v>
+      </c>
+      <c r="I11" s="9">
+        <v>0.0</v>
+      </c>
+      <c r="J11" s="9" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="C12" s="14">
+        <v>1.0</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="E12" s="9">
+        <v>3.43</v>
+      </c>
+      <c r="F12" s="9">
         <v>1.5</v>
       </c>
-      <c r="G8" s="13">
-        <v>0.0</v>
-      </c>
-      <c r="H8" s="13">
-        <v>0.0</v>
-      </c>
-      <c r="I8" s="13">
-        <v>0.0</v>
-      </c>
-      <c r="J8" s="13" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="13" t="s">
-        <v>50</v>
-      </c>
-      <c r="B9" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="C9" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="D9" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="E9" s="13">
+      <c r="G12" s="9">
+        <v>0.0</v>
+      </c>
+      <c r="H12" s="9">
+        <v>0.0</v>
+      </c>
+      <c r="I12" s="9">
+        <v>0.0</v>
+      </c>
+      <c r="J12" s="9" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="C13" s="9">
+        <v>1.2</v>
+      </c>
+      <c r="D13" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="E13" s="9">
         <v>3.43</v>
       </c>
-      <c r="F9" s="13">
+      <c r="F13" s="9">
         <v>1.5</v>
       </c>
-      <c r="G9" s="13">
+      <c r="G13" s="9">
         <v>8.0</v>
       </c>
-      <c r="H9" s="13">
+      <c r="H13" s="9">
         <v>4.0</v>
       </c>
-      <c r="I9" s="13">
+      <c r="I13" s="9">
         <v>5.0</v>
       </c>
-      <c r="J9" s="13" t="s">
+      <c r="J13" s="9" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="B10" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="C10" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="D10" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="E10" s="13">
+      <c r="B14" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="C14" s="9">
+        <v>1.2</v>
+      </c>
+      <c r="D14" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="E14" s="9">
         <v>6.86</v>
       </c>
-      <c r="F10" s="13">
-        <v>0.0</v>
-      </c>
-      <c r="G10" s="13">
+      <c r="F14" s="9">
+        <v>0.0</v>
+      </c>
+      <c r="G14" s="9">
         <v>8.0</v>
       </c>
-      <c r="H10" s="13">
+      <c r="H14" s="9">
         <v>4.0</v>
       </c>
-      <c r="I10" s="13">
+      <c r="I14" s="9">
         <v>5.0</v>
       </c>
-      <c r="J10" s="13" t="s">
+      <c r="J14" s="9" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="13" t="s">
-        <v>56</v>
-      </c>
-      <c r="B11" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="C11" s="13" t="s">
+      <c r="B15" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="E15" s="9">
+        <v>6.86</v>
+      </c>
+      <c r="F15" s="9">
+        <v>0.0</v>
+      </c>
+      <c r="G15" s="9">
+        <v>7.0</v>
+      </c>
+      <c r="H15" s="9">
+        <v>2.0</v>
+      </c>
+      <c r="I15" s="9">
+        <v>0.0</v>
+      </c>
+      <c r="J15" s="9" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="D11" s="13" t="s">
-        <v>40</v>
-      </c>
-      <c r="E11" s="13">
+      <c r="B16" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="C16" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="E16" s="9">
         <v>6.86</v>
       </c>
-      <c r="F11" s="13">
-        <v>0.0</v>
-      </c>
-      <c r="G11" s="13">
-        <v>7.0</v>
-      </c>
-      <c r="H11" s="13">
+      <c r="F16" s="9">
+        <v>0.0</v>
+      </c>
+      <c r="G16" s="9">
+        <v>13.0</v>
+      </c>
+      <c r="H16" s="9">
+        <v>0.0</v>
+      </c>
+      <c r="I16" s="9">
+        <v>8.0</v>
+      </c>
+      <c r="J16" s="9" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="B17" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="C17" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="D17" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="E17" s="9">
+        <v>6.86</v>
+      </c>
+      <c r="F17" s="9">
+        <v>0.0</v>
+      </c>
+      <c r="G17" s="9">
+        <v>13.0</v>
+      </c>
+      <c r="H17" s="9">
+        <v>0.0</v>
+      </c>
+      <c r="I17" s="9">
+        <v>8.0</v>
+      </c>
+      <c r="J17" s="9" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="B18" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="C18" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="D18" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="E18" s="9">
+        <v>3.2</v>
+      </c>
+      <c r="F18" s="9">
+        <v>0.0</v>
+      </c>
+      <c r="G18" s="15">
+        <v>13.0</v>
+      </c>
+      <c r="H18" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="I18" s="15">
+        <v>8.0</v>
+      </c>
+      <c r="J18" s="9" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="B19" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="C19" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="D19" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="E19" s="9">
+        <v>3.2</v>
+      </c>
+      <c r="F19" s="9">
+        <v>0.0</v>
+      </c>
+      <c r="G19" s="9">
+        <v>13.0</v>
+      </c>
+      <c r="H19" s="9">
+        <v>0.0</v>
+      </c>
+      <c r="I19" s="9">
+        <v>8.0</v>
+      </c>
+      <c r="J19" s="9" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="B20" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="C20" s="9">
+        <v>1.2</v>
+      </c>
+      <c r="D20" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="E20" s="9">
+        <v>3.43</v>
+      </c>
+      <c r="F20" s="9">
+        <v>3.43</v>
+      </c>
+      <c r="G20" s="9">
+        <v>8.0</v>
+      </c>
+      <c r="H20" s="9">
+        <v>4.0</v>
+      </c>
+      <c r="I20" s="9">
+        <v>8.0</v>
+      </c>
+      <c r="J20" s="9" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="B21" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="C21" s="9">
+        <v>1.2</v>
+      </c>
+      <c r="D21" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="E21" s="9">
+        <v>3.43</v>
+      </c>
+      <c r="F21" s="9">
+        <v>3.43</v>
+      </c>
+      <c r="G21" s="9">
+        <v>13.0</v>
+      </c>
+      <c r="H21" s="9">
+        <v>6.0</v>
+      </c>
+      <c r="I21" s="9">
+        <v>8.0</v>
+      </c>
+      <c r="J21" s="9" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="B22" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="C22" s="14">
         <v>2.0</v>
       </c>
-      <c r="I11" s="13">
-        <v>0.0</v>
-      </c>
-      <c r="J11" s="13" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="13" t="s">
-        <v>59</v>
-      </c>
-      <c r="B12" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="C12" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="D12" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="E12" s="13">
-        <v>6.86</v>
-      </c>
-      <c r="F12" s="13">
-        <v>0.0</v>
-      </c>
-      <c r="G12" s="13">
+      <c r="D22" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="E22" s="9">
+        <v>3.43</v>
+      </c>
+      <c r="F22" s="9">
+        <v>3.43</v>
+      </c>
+      <c r="G22" s="9">
         <v>13.0</v>
       </c>
-      <c r="H12" s="13">
-        <v>0.0</v>
-      </c>
-      <c r="I12" s="13">
+      <c r="H22" s="9">
+        <v>6.0</v>
+      </c>
+      <c r="I22" s="9">
         <v>8.0</v>
       </c>
-      <c r="J12" s="13" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="13" t="s">
-        <v>59</v>
-      </c>
-      <c r="B13" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="C13" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="D13" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="E13" s="13">
-        <v>6.86</v>
-      </c>
-      <c r="F13" s="13">
-        <v>0.0</v>
-      </c>
-      <c r="G13" s="13">
+      <c r="J22" s="9" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="B23" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="C23" s="14">
+        <v>2.0</v>
+      </c>
+      <c r="D23" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="E23" s="9">
+        <v>3.43</v>
+      </c>
+      <c r="F23" s="9">
+        <v>3.43</v>
+      </c>
+      <c r="G23" s="9">
+        <v>8.0</v>
+      </c>
+      <c r="H23" s="9">
+        <v>4.0</v>
+      </c>
+      <c r="I23" s="9">
+        <v>8.0</v>
+      </c>
+      <c r="J23" s="9" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="B24" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="C24" s="9">
+        <v>2.0</v>
+      </c>
+      <c r="D24" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="E24" s="9">
+        <v>3.43</v>
+      </c>
+      <c r="F24" s="9">
+        <v>3.43</v>
+      </c>
+      <c r="G24" s="16">
+        <v>8.0</v>
+      </c>
+      <c r="H24" s="16">
+        <v>4.0</v>
+      </c>
+      <c r="I24" s="16">
+        <v>8.0</v>
+      </c>
+      <c r="J24" s="16" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="B25" s="15" t="s">
+        <v>85</v>
+      </c>
+      <c r="C25" s="15">
+        <v>2.0</v>
+      </c>
+      <c r="D25" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="E25" s="18">
+        <v>3.43</v>
+      </c>
+      <c r="F25" s="18">
+        <v>3.43</v>
+      </c>
+      <c r="G25" s="17">
         <v>13.0</v>
       </c>
-      <c r="H13" s="13">
-        <v>0.0</v>
-      </c>
-      <c r="I13" s="13">
+      <c r="H25" s="17">
+        <v>6.0</v>
+      </c>
+      <c r="I25" s="17">
         <v>8.0</v>
       </c>
-      <c r="J13" s="13" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="B14" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="C14" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="D14" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="E14" s="13">
-        <v>3.2</v>
-      </c>
-      <c r="F14" s="13">
-        <v>0.0</v>
-      </c>
-      <c r="G14" s="15">
-        <v>13.0</v>
-      </c>
-      <c r="H14" s="15">
-        <v>0.0</v>
-      </c>
-      <c r="I14" s="15">
-        <v>8.0</v>
-      </c>
-      <c r="J14" s="13" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="B15" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="C15" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="D15" s="13" t="s">
-        <v>40</v>
-      </c>
-      <c r="E15" s="13">
-        <v>3.2</v>
-      </c>
-      <c r="F15" s="13">
-        <v>0.0</v>
-      </c>
-      <c r="G15" s="13">
-        <v>13.0</v>
-      </c>
-      <c r="H15" s="13">
-        <v>0.0</v>
-      </c>
-      <c r="I15" s="13">
-        <v>8.0</v>
-      </c>
-      <c r="J15" s="13" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="13" t="s">
-        <v>65</v>
-      </c>
-      <c r="B16" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="C16" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="D16" s="13" t="s">
-        <v>40</v>
-      </c>
-      <c r="E16" s="13">
+      <c r="J25" s="17" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="15" t="s">
+        <v>75</v>
+      </c>
+      <c r="B26" s="15" t="s">
+        <v>85</v>
+      </c>
+      <c r="C26" s="15">
+        <v>1.0</v>
+      </c>
+      <c r="D26" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="E26" s="18">
         <v>3.43</v>
       </c>
-      <c r="F16" s="13">
+      <c r="F26" s="18">
         <v>3.43</v>
       </c>
-      <c r="G16" s="13">
-        <v>8.0</v>
-      </c>
-      <c r="H16" s="13">
-        <v>4.0</v>
-      </c>
-      <c r="I16" s="13">
-        <v>8.0</v>
-      </c>
-      <c r="J16" s="13" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="13" t="s">
-        <v>67</v>
-      </c>
-      <c r="B17" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="C17" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="D17" s="13" t="s">
-        <v>40</v>
-      </c>
-      <c r="E17" s="13">
+      <c r="G26" s="17">
+        <v>0.0</v>
+      </c>
+      <c r="H26" s="17">
+        <v>0.0</v>
+      </c>
+      <c r="I26" s="17">
+        <v>0.0</v>
+      </c>
+      <c r="J26" s="17" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="15" t="s">
+        <v>77</v>
+      </c>
+      <c r="B27" s="15" t="s">
+        <v>85</v>
+      </c>
+      <c r="C27" s="15">
+        <v>1.0</v>
+      </c>
+      <c r="D27" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="E27" s="18">
         <v>3.43</v>
       </c>
-      <c r="F17" s="13">
+      <c r="F27" s="18">
         <v>3.43</v>
       </c>
-      <c r="G17" s="13">
-        <v>13.0</v>
-      </c>
-      <c r="H17" s="13">
-        <v>6.0</v>
-      </c>
-      <c r="I17" s="13">
-        <v>8.0</v>
-      </c>
-      <c r="J17" s="13" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="13" t="s">
-        <v>69</v>
-      </c>
-      <c r="B18" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="C18" s="14">
-        <v>2.0</v>
-      </c>
-      <c r="D18" s="13" t="s">
-        <v>40</v>
-      </c>
-      <c r="E18" s="13">
-        <v>3.43</v>
-      </c>
-      <c r="F18" s="13">
-        <v>3.43</v>
-      </c>
-      <c r="G18" s="13">
-        <v>13.0</v>
-      </c>
-      <c r="H18" s="13">
-        <v>6.0</v>
-      </c>
-      <c r="I18" s="13">
-        <v>8.0</v>
-      </c>
-      <c r="J18" s="13" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="13" t="s">
-        <v>71</v>
-      </c>
-      <c r="B19" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="C19" s="14">
-        <v>2.0</v>
-      </c>
-      <c r="D19" s="13" t="s">
-        <v>40</v>
-      </c>
-      <c r="E19" s="13">
-        <v>3.43</v>
-      </c>
-      <c r="F19" s="13">
-        <v>3.43</v>
-      </c>
-      <c r="G19" s="13">
-        <v>8.0</v>
-      </c>
-      <c r="H19" s="13">
-        <v>4.0</v>
-      </c>
-      <c r="I19" s="13">
-        <v>8.0</v>
-      </c>
-      <c r="J19" s="13" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="13" t="s">
-        <v>73</v>
-      </c>
-      <c r="B20" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="C20" s="13">
-        <v>2.0</v>
-      </c>
-      <c r="D20" s="16" t="s">
-        <v>31</v>
-      </c>
-      <c r="E20" s="13">
-        <v>3.43</v>
-      </c>
-      <c r="F20" s="13">
-        <v>3.43</v>
-      </c>
-      <c r="G20" s="16">
-        <v>8.0</v>
-      </c>
-      <c r="H20" s="16">
-        <v>4.0</v>
-      </c>
-      <c r="I20" s="16">
-        <v>8.0</v>
-      </c>
-      <c r="J20" s="16" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="15" t="s">
-        <v>75</v>
-      </c>
-      <c r="B21" s="15" t="s">
-        <v>39</v>
-      </c>
-      <c r="C21" s="15">
-        <v>2.0</v>
-      </c>
-      <c r="D21" s="17" t="s">
-        <v>31</v>
-      </c>
-      <c r="E21" s="18">
-        <v>3.43</v>
-      </c>
-      <c r="F21" s="18">
-        <v>3.43</v>
-      </c>
-      <c r="G21" s="17">
-        <v>13.0</v>
-      </c>
-      <c r="H21" s="17">
-        <v>6.0</v>
-      </c>
-      <c r="I21" s="17">
-        <v>8.0</v>
-      </c>
-      <c r="J21" s="17" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="15" t="s">
-        <v>77</v>
-      </c>
-      <c r="B22" s="15" t="s">
-        <v>39</v>
-      </c>
-      <c r="C22" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="D22" s="17" t="s">
-        <v>31</v>
-      </c>
-      <c r="E22" s="18">
-        <v>3.43</v>
-      </c>
-      <c r="F22" s="18">
-        <v>3.43</v>
-      </c>
-      <c r="G22" s="17">
-        <v>0.0</v>
-      </c>
-      <c r="H22" s="17">
-        <v>0.0</v>
-      </c>
-      <c r="I22" s="17">
-        <v>0.0</v>
-      </c>
-      <c r="J22" s="17" t="s">
+      <c r="G27" s="17">
+        <v>0.0</v>
+      </c>
+      <c r="H27" s="17">
+        <v>0.0</v>
+      </c>
+      <c r="I27" s="17">
+        <v>0.0</v>
+      </c>
+      <c r="J27" s="17" t="s">
         <v>78</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="15" t="s">
-        <v>79</v>
-      </c>
-      <c r="B23" s="15" t="s">
-        <v>39</v>
-      </c>
-      <c r="C23" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="D23" s="17" t="s">
-        <v>31</v>
-      </c>
-      <c r="E23" s="18">
-        <v>3.43</v>
-      </c>
-      <c r="F23" s="18">
-        <v>3.43</v>
-      </c>
-      <c r="G23" s="17">
-        <v>0.0</v>
-      </c>
-      <c r="H23" s="17">
-        <v>0.0</v>
-      </c>
-      <c r="I23" s="17">
-        <v>0.0</v>
-      </c>
-      <c r="J23" s="17" t="s">
-        <v>80</v>
       </c>
     </row>
   </sheetData>

</xml_diff>